<commit_message>
NDT report: DAVIT CRANES 25380/ndt_report_20260303_1312.md
</commit_message>
<xml_diff>
--- a/DAVIT CRANES 25380/ndt_report_20260303_1312.xlsx
+++ b/DAVIT CRANES 25380/ndt_report_20260303_1312.xlsx
@@ -3058,7 +3058,7 @@
       </c>
       <c r="C103" s="42" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>26/02/2026</t>
         </is>
       </c>
       <c r="D103" s="106" t="n"/>
@@ -3068,7 +3068,7 @@
       </c>
       <c r="F103" s="38" t="inlineStr">
         <is>
-          <t>- Magnetic Particle Testing (MT) — per EN ISO 17638; - Penetrant Testing (PT) — per EN ISO 3452-1; - Ultrasonic Testing (UT) — per EN ISO 17640</t>
+          <t>00:38 — Jan Verheyen: Veel plezier daar, just de wieken op de brug gezien, waren er 3 &lt;Dit bericht i; The image displays a fillet weld on a davit crane component (Undercover op nr 30, project 25380 Seas; The davit crane components exhibit a grey industrial coating, likely hot-dip galvanization. Minor su</t>
         </is>
       </c>
       <c r="G103" s="104" t="n"/>
@@ -3107,21 +3107,13 @@
           <t xml:space="preserve">Date </t>
         </is>
       </c>
-      <c r="C106" s="42" t="inlineStr">
-        <is>
-          <t>26/02/2026</t>
-        </is>
-      </c>
+      <c r="C106" s="42" t="n"/>
       <c r="D106" s="106" t="n"/>
       <c r="E106" s="37">
         <f>IF(F106="","","→")</f>
         <v/>
       </c>
-      <c r="F106" s="38" t="inlineStr">
-        <is>
-          <t>00:38 — Jan Verheyen: Veel plezier daar, just de wieken op de brug gezien, waren er 3 &lt;Dit bericht i; The image displays a fillet weld on a davit crane component (Undercover op nr 30, project 25380 Seas; The davit crane components exhibit a grey industrial coating, likely hot-dip galvanization. Minor su</t>
-        </is>
-      </c>
+      <c r="F106" s="38" t="n"/>
       <c r="G106" s="104" t="n"/>
     </row>
     <row r="107" ht="17.25" customHeight="1">
@@ -3158,21 +3150,13 @@
           <t xml:space="preserve">Date </t>
         </is>
       </c>
-      <c r="C109" s="42" t="inlineStr">
-        <is>
-          <t>03/03/2026</t>
-        </is>
-      </c>
+      <c r="C109" s="42" t="n"/>
       <c r="D109" s="106" t="n"/>
       <c r="E109" s="37">
         <f>IF(F109="","","→")</f>
         <v/>
       </c>
-      <c r="F109" s="38" t="inlineStr">
-        <is>
-          <t>- No specific NDT methods recorded; (No NDT-related worklog entries found); [To be completed by inspector]</t>
-        </is>
-      </c>
+      <c r="F109" s="38" t="n"/>
       <c r="G109" s="104" t="n"/>
     </row>
     <row r="110" ht="17.25" customHeight="1">
@@ -3209,21 +3193,13 @@
           <t xml:space="preserve">Date </t>
         </is>
       </c>
-      <c r="C112" s="42" t="inlineStr">
-        <is>
-          <t>02/03/2026</t>
-        </is>
-      </c>
+      <c r="C112" s="42" t="n"/>
       <c r="D112" s="106" t="n"/>
       <c r="E112" s="37">
         <f>IF(F112="","","→")</f>
         <v/>
       </c>
-      <c r="F112" s="38" t="inlineStr">
-        <is>
-          <t>- No specific NDT methods recorded; (No NDT-related worklog entries found); [To be completed by inspector]</t>
-        </is>
-      </c>
+      <c r="F112" s="38" t="n"/>
       <c r="G112" s="104" t="n"/>
     </row>
     <row r="113" ht="17.25" customHeight="1">
@@ -3260,21 +3236,13 @@
           <t xml:space="preserve">Date </t>
         </is>
       </c>
-      <c r="C115" s="42" t="inlineStr">
-        <is>
-          <t>01/03/2026</t>
-        </is>
-      </c>
+      <c r="C115" s="42" t="n"/>
       <c r="D115" s="106" t="n"/>
       <c r="E115" s="37">
         <f>IF(F115="","","→")</f>
         <v/>
       </c>
-      <c r="F115" s="38" t="inlineStr">
-        <is>
-          <t>- No specific NDT methods recorded; (No NDT-related worklog entries found); [To be completed by inspector]</t>
-        </is>
-      </c>
+      <c r="F115" s="38" t="n"/>
       <c r="G115" s="104" t="n"/>
     </row>
     <row r="116" ht="17.25" customHeight="1">

</xml_diff>